<commit_message>
feat: add sidebar navigation and default relocation
</commit_message>
<xml_diff>
--- a/jobs_master.xlsx
+++ b/jobs_master.xlsx
@@ -2379,7 +2379,11 @@
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>resumes/SujanDora_resume_Dexian_v20260129_185044.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">

</xml_diff>